<commit_message>
update income definitions and min wage compliance variables
</commit_message>
<xml_diff>
--- a/codes.xlsx
+++ b/codes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Research Projects\Frank Chapter 3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{799326DC-0F1F-45A9-8766-3196F1F0BA3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE6E27A1-40EE-4ACC-8C30-E7A54AE3E1C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{97F336A6-7C7A-4FB8-8073-41CBB847BCE1}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="138">
   <si>
     <t>total_income_primary</t>
   </si>
@@ -231,9 +231,6 @@
     <t>This represents total value of renumerations for primary job. Includes cash, benefits value and in kind pay</t>
   </si>
   <si>
-    <t>Definition</t>
-  </si>
-  <si>
     <t>Dataset Variable</t>
   </si>
   <si>
@@ -241,6 +238,207 @@
   </si>
   <si>
     <t>CATEGORIA_PRINCIPAL</t>
+  </si>
+  <si>
+    <t>Survey Data Variable</t>
+  </si>
+  <si>
+    <t>comission_income_primary</t>
+  </si>
+  <si>
+    <t>tips_income_primary</t>
+  </si>
+  <si>
+    <t>overtime_income_primary</t>
+  </si>
+  <si>
+    <t>other_income_primary</t>
+  </si>
+  <si>
+    <t>COMISIONES</t>
+  </si>
+  <si>
+    <t>PROPINAS</t>
+  </si>
+  <si>
+    <t>HORAS_EXTRA</t>
+  </si>
+  <si>
+    <t>OTROS_PAGOS</t>
+  </si>
+  <si>
+    <t>vacation_benefit_primary</t>
+  </si>
+  <si>
+    <t>bonus_benefit_primary</t>
+  </si>
+  <si>
+    <t>christmas_benefit_primary</t>
+  </si>
+  <si>
+    <t>senority_benefit_primary</t>
+  </si>
+  <si>
+    <t>other_benefit_primary</t>
+  </si>
+  <si>
+    <t>food_inkind_primary</t>
+  </si>
+  <si>
+    <t>housing_inkind_primary</t>
+  </si>
+  <si>
+    <t>transport_inkind_primary</t>
+  </si>
+  <si>
+    <t>gas_inkind_primary</t>
+  </si>
+  <si>
+    <t>cell_inkind_primary</t>
+  </si>
+  <si>
+    <t>other_inkind_primary</t>
+  </si>
+  <si>
+    <t>ESPECIE_ALIMENTOS</t>
+  </si>
+  <si>
+    <t>ESPECIE_VIVIENDA</t>
+  </si>
+  <si>
+    <t>ESPECIE_TRANSPORTE</t>
+  </si>
+  <si>
+    <t>ESPECIE_COMBUSTIBLE</t>
+  </si>
+  <si>
+    <t>ESPECIE_CELULAR</t>
+  </si>
+  <si>
+    <t>OTROS_ESPECIE</t>
+  </si>
+  <si>
+    <t>BONO_VACACIONES</t>
+  </si>
+  <si>
+    <t>BONIFICACIONES</t>
+  </si>
+  <si>
+    <t>REGALIA_PASCUAL</t>
+  </si>
+  <si>
+    <t>INCENTIVO_ANTIGUEDAD</t>
+  </si>
+  <si>
+    <t>OTROS_BENEFICIOS</t>
+  </si>
+  <si>
+    <t>Units</t>
+  </si>
+  <si>
+    <t>independent_benefit_primary</t>
+  </si>
+  <si>
+    <t>independent_inkind_primary</t>
+  </si>
+  <si>
+    <t>CONSUMO_BIENES</t>
+  </si>
+  <si>
+    <t>ESPECIE_INDEPENDIENTES</t>
+  </si>
+  <si>
+    <t>other_income_secondary</t>
+  </si>
+  <si>
+    <t>OTROS_PAGOS_SECUN</t>
+  </si>
+  <si>
+    <t>benefits_income_secondary</t>
+  </si>
+  <si>
+    <t>inkind_secondary</t>
+  </si>
+  <si>
+    <t>independent_benefit_secondary</t>
+  </si>
+  <si>
+    <t>independent_inkind_secondary</t>
+  </si>
+  <si>
+    <t>ESPECIE_INDEPENDIENTES_SECUN</t>
+  </si>
+  <si>
+    <t>CONSUMO_BIENES_SECUN</t>
+  </si>
+  <si>
+    <t>total_comp_primary</t>
+  </si>
+  <si>
+    <t>nonsalary_income_secondary</t>
+  </si>
+  <si>
+    <t>total_comp_secondary</t>
+  </si>
+  <si>
+    <t>INGRESO_ASALARIADO + COMISIONES + PROPINAS + HORAS_EXTRA + OTROS_PAGOS + INGRESO_INDEPENDIENTES</t>
+  </si>
+  <si>
+    <t>INGRESO_ASALARIADO + COMISIONES</t>
+  </si>
+  <si>
+    <t>INGRESO_ASALARIADO_SECUN + OTROS_PAGOS_SECUN + INGRESO_INDEPENDIENTES_SECUN</t>
+  </si>
+  <si>
+    <t>OTROS_BENEFICIOS_SECUN + CONSUMO_BIENES_SECUN</t>
+  </si>
+  <si>
+    <t>PAGO_ESPECIE_SECUN + ESPECIE_INDEPENDIENTES_SECUN</t>
+  </si>
+  <si>
+    <t>INGRESO_ASALARIADO_SECUN + OTROS_PAGOS_SECUN + INGRESO_INDEPENDIENTES_SECUN + OTROS_BENEFICIOS_SECUN + CONSUMO_BIENES_SECUN + PAGO_ESPECIE_SECUN + ESPECIE_INDEPENDIENTES_SECUN</t>
+  </si>
+  <si>
+    <t>BONO_VACACIONES + BONIFICACIONES + REGALIA_PASCUAL + INCENTIVO_ANTIGUEDAD + OTROS_BENEFICIOS + CONSUMO_BIENES</t>
+  </si>
+  <si>
+    <t>ESPECIE_ALIMENTOS + ESPECIE_VIVIENDA + ESPECIE_TRANSPORTE + ESPECIE_COMBUSTIBLE +  ESPECIE_CELULAR + OTROS_ESPECIE + ESPECIE_INDEPENDIENTES</t>
+  </si>
+  <si>
+    <t>INGRESO_ASALARIADO + COMISIONES + PROPINAS + HORAS_EXTRA + OTROS_PAGOS + INGRESO_INDEPENDIENTES + BONO_VACACIONES + BONIFICACIONES + REGALIA_PASCUAL + INCENTIVO_ANTIGUEDAD + OTROS_BENEFICIOS + CONSUMO_BIENES + ESPECIE_ALIMENTOS + ESPECIE_VIVIENDA + ESPECIE_TRANSPORTE + ESPECIE_COMBUSTIBLE +  ESPECIE_CELULAR + OTROS_ESPECIE + ESPECIE_INDEPENDIENTES</t>
+  </si>
+  <si>
+    <t>benefits_total</t>
+  </si>
+  <si>
+    <t>salary_total</t>
+  </si>
+  <si>
+    <t>nonsalary_total</t>
+  </si>
+  <si>
+    <t>inkind_total</t>
+  </si>
+  <si>
+    <t>INGRESO_ASALARIADO + INGRESO_ASALARIADO_SECUN</t>
+  </si>
+  <si>
+    <t>COMISIONES + PROPINAS + HORAS_EXTRA + OTROS_PAGOS + INGRESO_INDEPENDIENTES + OTROS_PAGOS_SECUN + INGRESO_INDEPENDIENTES_SECUN</t>
+  </si>
+  <si>
+    <t>income_total</t>
+  </si>
+  <si>
+    <t>INGRESO_ASALARIADO + INGRESO_ASALARIADO_SECUN + COMISIONES + PROPINAS + HORAS_EXTRA + OTROS_PAGOS + INGRESO_INDEPENDIENTES + OTROS_PAGOS_SECUN + INGRESO_INDEPENDIENTES_SECUN</t>
+  </si>
+  <si>
+    <t>BONO_VACACIONES + BONIFICACIONES + REGALIA_PASCUAL + INCENTIVO_ANTIGUEDAD + OTROS_BENEFICIOS + CONSUMO_BIENES + OTROS_BENEFICIOS_SECUN + CONSUMO_BIENES_SECUN</t>
+  </si>
+  <si>
+    <t>ESPECIE_ALIMENTOS + ESPECIE_VIVIENDA + ESPECIE_TRANSPORTE + ESPECIE_COMBUSTIBLE +  ESPECIE_CELULAR + OTROS_ESPECIE + ESPECIE_INDEPENDIENTES + PAGO_ESPECIE_SECUN + ESPECIE_INDEPENDIENTES_SECUN</t>
+  </si>
+  <si>
+    <t>INGRESO_INDEPENDIENTES + INGRESO_INDEPENDIENTES_SECUN</t>
   </si>
 </sst>
 </file>
@@ -297,7 +495,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -308,6 +506,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -622,7 +823,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2534CD19-0EFF-4C7D-B6DA-E9A67839C40C}">
-  <dimension ref="A3:I45"/>
+  <dimension ref="A3:J106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="39.5703125" customWidth="1"/>
@@ -630,18 +831,21 @@
     <col min="9" max="9" width="73" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="7:10" x14ac:dyDescent="0.25">
       <c r="G3" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J3" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" spans="7:10" x14ac:dyDescent="0.25">
       <c r="G4" t="s">
         <v>7</v>
       </c>
@@ -652,308 +856,652 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="7:10" x14ac:dyDescent="0.25">
       <c r="G5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="G6" t="s">
+        <v>73</v>
+      </c>
+      <c r="H6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="G7" t="s">
+        <v>74</v>
+      </c>
+      <c r="H7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="G8" t="s">
+        <v>75</v>
+      </c>
+      <c r="H8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="G10" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="G11" t="s">
+        <v>103</v>
+      </c>
+      <c r="H11" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="12" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="G12" t="s">
+        <v>104</v>
+      </c>
+      <c r="H12" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="14" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="G14" t="s">
+        <v>80</v>
+      </c>
+      <c r="H14" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="G15" t="s">
+        <v>81</v>
+      </c>
+      <c r="H15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="G16" t="s">
+        <v>82</v>
+      </c>
+      <c r="H16" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="17" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G17" t="s">
+        <v>83</v>
+      </c>
+      <c r="H17" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G18" t="s">
+        <v>84</v>
+      </c>
+      <c r="H18" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G20" t="s">
+        <v>85</v>
+      </c>
+      <c r="H20" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="21" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G21" t="s">
+        <v>86</v>
+      </c>
+      <c r="H21" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="22" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G22" t="s">
+        <v>87</v>
+      </c>
+      <c r="H22" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="23" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G23" t="s">
+        <v>88</v>
+      </c>
+      <c r="H23" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="24" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G24" t="s">
+        <v>89</v>
+      </c>
+      <c r="H24" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="25" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G25" t="s">
+        <v>90</v>
+      </c>
+      <c r="H25" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="27" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G27" t="s">
+        <v>25</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" spans="7:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="G28" t="s">
+        <v>0</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="29" spans="7:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="G29" t="s">
+        <v>1</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="30" spans="7:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="G30" t="s">
+        <v>2</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="31" spans="7:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="G31" t="s">
+        <v>115</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="32" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G32" t="s">
+        <v>3</v>
+      </c>
+      <c r="H32" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="35" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G35" t="s">
         <v>8</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H35" t="s">
         <v>22</v>
       </c>
-      <c r="I5" t="s">
+    </row>
+    <row r="36" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G36" t="s">
+        <v>107</v>
+      </c>
+      <c r="H36" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="38" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G38" t="s">
+        <v>109</v>
+      </c>
+      <c r="H38" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="39" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G39" t="s">
+        <v>110</v>
+      </c>
+      <c r="H39" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="41" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G41" t="s">
+        <v>9</v>
+      </c>
+      <c r="H41" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="42" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G42" t="s">
+        <v>111</v>
+      </c>
+      <c r="H42" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="43" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G43" t="s">
+        <v>112</v>
+      </c>
+      <c r="H43" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="45" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G45" t="s">
+        <v>116</v>
+      </c>
+      <c r="H45" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="46" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G46" t="s">
+        <v>11</v>
+      </c>
+      <c r="H46" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="47" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G47" t="s">
+        <v>12</v>
+      </c>
+      <c r="H47" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="48" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G48" t="s">
+        <v>13</v>
+      </c>
+      <c r="H48" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="49" spans="7:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="G49" t="s">
+        <v>117</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="52" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G52" t="s">
+        <v>128</v>
+      </c>
+      <c r="H52" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="53" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G53" t="s">
+        <v>129</v>
+      </c>
+      <c r="H53" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="54" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G54" t="s">
+        <v>133</v>
+      </c>
+      <c r="H54" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="55" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G55" t="s">
+        <v>127</v>
+      </c>
+      <c r="H55" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="56" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G56" t="s">
+        <v>130</v>
+      </c>
+      <c r="H56" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="58" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G58" t="s">
+        <v>18</v>
+      </c>
+      <c r="H58" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="59" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G59" t="s">
+        <v>19</v>
+      </c>
+      <c r="H59" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G66" t="s">
+        <v>8</v>
+      </c>
+      <c r="H66" t="s">
+        <v>22</v>
+      </c>
+      <c r="I66" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G6" s="3" t="s">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G67" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H67" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I67" s="3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G9" t="s">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G70" t="s">
         <v>6</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H70" t="s">
         <v>24</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I70" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>3</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G71" t="s">
         <v>9</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H71" t="s">
         <v>23</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I71" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
         <v>4</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G72" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="H72" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="I72" s="3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="G13" t="s">
+    <row r="74" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="G74" t="s">
         <v>25</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H74" t="s">
         <v>27</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="I74" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="G14" t="s">
+    <row r="75" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="G75" t="s">
         <v>26</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H75" t="s">
         <v>28</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="I75" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G15" s="3" t="s">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G76" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="H15" s="3" t="s">
+      <c r="H76" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="I76" s="4" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I16" s="2"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I17" s="2"/>
-    </row>
-    <row r="18" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G18" s="3" t="s">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I77" s="2"/>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I78" s="2"/>
+    </row>
+    <row r="79" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G79" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="H18" s="3" t="s">
+      <c r="H79" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="I79" s="4" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="G19" s="3" t="s">
+    <row r="80" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="G80" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="H19" s="3" t="s">
+      <c r="H80" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="I80" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G20" s="3" t="s">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G81" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="H20" s="3" t="s">
+      <c r="H81" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="I20" s="4" t="s">
+      <c r="I81" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I21" s="2"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I22" s="2"/>
-    </row>
-    <row r="23" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="G23" t="s">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I82" s="2"/>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I83" s="2"/>
+    </row>
+    <row r="84" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="G84" t="s">
         <v>1</v>
       </c>
-      <c r="H23" t="s">
+      <c r="H84" t="s">
         <v>51</v>
       </c>
-      <c r="I23" s="2" t="s">
+      <c r="I84" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="G24" t="s">
+    <row r="85" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="G85" t="s">
         <v>12</v>
       </c>
-      <c r="H24" t="s">
+      <c r="H85" t="s">
         <v>50</v>
       </c>
-      <c r="I24" s="2" t="s">
+      <c r="I85" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G25" t="s">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G86" t="s">
         <v>16</v>
       </c>
-      <c r="H25" t="s">
+      <c r="H86" t="s">
         <v>54</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="I86" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>10</v>
       </c>
-      <c r="I26" s="2"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="I87" s="2"/>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>11</v>
       </c>
-      <c r="I27" s="2"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G28" t="s">
+      <c r="I88" s="2"/>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G89" t="s">
         <v>2</v>
       </c>
-      <c r="H28" t="s">
+      <c r="H89" t="s">
         <v>56</v>
       </c>
-      <c r="I28" s="2"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="I89" s="2"/>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>13</v>
       </c>
-      <c r="G29" t="s">
+      <c r="G90" t="s">
         <v>13</v>
       </c>
-      <c r="H29" t="s">
+      <c r="H90" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G30" s="5" t="s">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G91" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H30" s="5" t="s">
+      <c r="H91" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="I30" s="5"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="I91" s="5"/>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
         <v>15</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G94" t="s">
         <v>19</v>
       </c>
-      <c r="H33" t="s">
+      <c r="H94" t="s">
         <v>59</v>
       </c>
-      <c r="I33" t="s">
+      <c r="I94" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
         <v>16</v>
       </c>
-      <c r="G34" t="s">
+      <c r="G95" t="s">
         <v>20</v>
       </c>
-      <c r="I34" t="s">
+      <c r="I95" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G38" t="s">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G99" t="s">
         <v>3</v>
       </c>
-      <c r="H38" t="s">
+      <c r="H99" t="s">
         <v>63</v>
       </c>
-      <c r="I38" t="s">
+      <c r="I99" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>19</v>
       </c>
-      <c r="G39" t="s">
+      <c r="G100" t="s">
         <v>4</v>
       </c>
-      <c r="H39" t="s">
+      <c r="H100" t="s">
         <v>62</v>
       </c>
-      <c r="I39" t="s">
+      <c r="I100" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G40" t="s">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G101" t="s">
         <v>5</v>
       </c>
-      <c r="H40" t="s">
+      <c r="H101" t="s">
         <v>66</v>
       </c>
-      <c r="I40" t="s">
+      <c r="I101" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G44" t="s">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G105" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G106" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G45" t="s">
-        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>